<commit_message>
add route manager for end to end flow
</commit_message>
<xml_diff>
--- a/src/test/resources/ExcelResultsFolder/Cards.xlsx
+++ b/src/test/resources/ExcelResultsFolder/Cards.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\git\Integration\src\test\resources\ExcelResultsFolder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA18E017-9ED3-463E-908A-0A5FBD8E1EE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{536182D8-FB84-49C2-B300-348AD435CEC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="77">
   <si>
     <t>Matrix</t>
   </si>
@@ -244,22 +244,10 @@
     <t>euroexchange</t>
   </si>
   <si>
-    <t>AED</t>
-  </si>
-  <si>
-    <t>4456530000001096</t>
-  </si>
-  <si>
     <t>02/29</t>
   </si>
   <si>
     <t>123</t>
-  </si>
-  <si>
-    <t>telr</t>
-  </si>
-  <si>
-    <t>5200000000001096</t>
   </si>
   <si>
     <t>CAD</t>
@@ -707,7 +695,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A047734-60A8-451A-B92F-500542A01A48}">
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.81640625" customWidth="1"/>
@@ -865,7 +853,7 @@
         <v>500</v>
       </c>
       <c r="O3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.35">
@@ -873,22 +861,22 @@
         <v>17</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>67</v>
+        <v>18</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" t="s">
+        <v>0</v>
+      </c>
+      <c r="F4" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="G4" t="s">
         <v>68</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="E4" t="s">
-        <v>70</v>
-      </c>
-      <c r="F4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" t="s">
-        <v>66</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>56</v>
@@ -900,7 +888,7 @@
         <v>54</v>
       </c>
       <c r="K4" t="s">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="L4" s="4">
         <v>10</v>
@@ -912,7 +900,7 @@
         <v>100</v>
       </c>
       <c r="O4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.35">
@@ -920,22 +908,22 @@
         <v>17</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="E5" t="s">
-        <v>70</v>
-      </c>
       <c r="F5" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="G5" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H5" s="4" t="s">
         <v>56</v>
@@ -947,7 +935,7 @@
         <v>54</v>
       </c>
       <c r="K5" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="L5" s="4">
         <v>10</v>
@@ -956,10 +944,10 @@
         <v>100</v>
       </c>
       <c r="N5" s="4">
-        <v>100</v>
+        <v>55.3</v>
       </c>
       <c r="O5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.35">
@@ -967,19 +955,19 @@
         <v>17</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>18</v>
+        <v>74</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>19</v>
+        <v>66</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E6" t="s">
-        <v>0</v>
-      </c>
-      <c r="F6" s="15" t="s">
-        <v>73</v>
+        <v>67</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="F6" t="s">
+        <v>12</v>
       </c>
       <c r="G6" t="s">
         <v>72</v>
@@ -993,114 +981,20 @@
       <c r="J6" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="K6" t="s">
-        <v>50</v>
+      <c r="K6" s="16" t="s">
+        <v>76</v>
       </c>
       <c r="L6" s="4">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="M6" s="4">
-        <v>100</v>
+        <v>900</v>
       </c>
       <c r="N6" s="4">
-        <v>100</v>
+        <v>569</v>
       </c>
       <c r="O6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="F7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G7" t="s">
-        <v>76</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="I7" t="s">
-        <v>46</v>
-      </c>
-      <c r="J7" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="K7" t="s">
-        <v>77</v>
-      </c>
-      <c r="L7" s="4">
-        <v>10</v>
-      </c>
-      <c r="M7" s="4">
-        <v>100</v>
-      </c>
-      <c r="N7" s="4">
-        <v>55.3</v>
-      </c>
-      <c r="O7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="F8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G8" t="s">
-        <v>76</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="I8" t="s">
-        <v>46</v>
-      </c>
-      <c r="J8" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="K8" s="16" t="s">
-        <v>80</v>
-      </c>
-      <c r="L8" s="4">
-        <v>10</v>
-      </c>
-      <c r="M8" s="4">
-        <v>100</v>
-      </c>
-      <c r="N8" s="4">
-        <v>55.3</v>
-      </c>
-      <c r="O8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1226,7 +1120,7 @@
         <v>500</v>
       </c>
       <c r="P2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.35">
@@ -1276,7 +1170,7 @@
         <v>500</v>
       </c>
       <c r="P3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.35">
@@ -1376,7 +1270,7 @@
         <v>500</v>
       </c>
       <c r="P5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.35">
@@ -1476,7 +1370,7 @@
         <v>10</v>
       </c>
       <c r="P7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
change random data like email
</commit_message>
<xml_diff>
--- a/src/test/resources/ExcelResultsFolder/Cards.xlsx
+++ b/src/test/resources/ExcelResultsFolder/Cards.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\git\Integration\src\test\resources\ExcelResultsFolder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E3315B4-470B-40F5-808B-4A6D3DA939C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BCA6DBC-46D8-4B60-98CE-1F87700A9F4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -966,7 +966,7 @@
         <v>55.3</v>
       </c>
       <c r="O5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
run for all test
</commit_message>
<xml_diff>
--- a/src/test/resources/ExcelResultsFolder/Cards.xlsx
+++ b/src/test/resources/ExcelResultsFolder/Cards.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\git\Integration\src\test\resources\ExcelResultsFolder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A310ABE-7A3C-42CD-8FE1-9B1FA075DE9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61BB6613-052D-4C7B-AFF9-6486A050F656}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1081,7 +1081,7 @@
         <v>569</v>
       </c>
       <c r="O7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.35">
@@ -1128,7 +1128,7 @@
         <v>569</v>
       </c>
       <c r="O8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.35">
@@ -1175,7 +1175,7 @@
         <v>569</v>
       </c>
       <c r="O9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.35">
@@ -1222,7 +1222,7 @@
         <v>569</v>
       </c>
       <c r="O10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.35">
@@ -1269,7 +1269,7 @@
         <v>569</v>
       </c>
       <c r="O11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.35">
@@ -1316,7 +1316,7 @@
         <v>569</v>
       </c>
       <c r="O12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
run for trustpayments token
</commit_message>
<xml_diff>
--- a/src/test/resources/ExcelResultsFolder/Cards.xlsx
+++ b/src/test/resources/ExcelResultsFolder/Cards.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\git\Integration\src\test\resources\ExcelResultsFolder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61BB6613-052D-4C7B-AFF9-6486A050F656}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFEC88B9-BF7F-47E0-B116-17A27B86481F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1034,7 +1034,7 @@
         <v>569</v>
       </c>
       <c r="O6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.35">
@@ -1081,7 +1081,7 @@
         <v>569</v>
       </c>
       <c r="O7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.35">
@@ -1128,7 +1128,7 @@
         <v>569</v>
       </c>
       <c r="O8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.35">
@@ -1175,7 +1175,7 @@
         <v>569</v>
       </c>
       <c r="O9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
run for unicorn 3ds page
</commit_message>
<xml_diff>
--- a/src/test/resources/ExcelResultsFolder/Cards.xlsx
+++ b/src/test/resources/ExcelResultsFolder/Cards.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\git\Integration\src\test\resources\ExcelResultsFolder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9455579D-653C-447F-82E1-B64D0D600429}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93E48FA4-4297-43D1-8D3F-D93E833437AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -334,7 +334,7 @@
     <t>4100000000005000</t>
   </si>
   <si>
-    <t>unicornpayment3ds</t>
+    <t>unicornpaymentds</t>
   </si>
 </sst>
 </file>
@@ -1387,7 +1387,7 @@
         <v>569</v>
       </c>
       <c r="O13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
cc avenue is done
</commit_message>
<xml_diff>
--- a/src/test/resources/ExcelResultsFolder/Cards.xlsx
+++ b/src/test/resources/ExcelResultsFolder/Cards.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\git\Integration\src\test\resources\ExcelResultsFolder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{584731D3-684E-4EDD-AA21-197729E55E8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B520A3B-5D98-49DA-9DFD-555F41B3130E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="107">
   <si>
     <t>Matrix</t>
   </si>
@@ -362,6 +362,9 @@
   </si>
   <si>
     <t>5123450000000008</t>
+  </si>
+  <si>
+    <t>4242424242424242</t>
   </si>
 </sst>
 </file>
@@ -786,7 +789,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A047734-60A8-451A-B92F-500542A01A48}">
-  <dimension ref="A1:O18"/>
+  <dimension ref="A1:O19"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.81640625" customWidth="1"/>
@@ -1555,11 +1558,58 @@
         <v>369</v>
       </c>
       <c r="O16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>104</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="E17" t="s">
+        <v>102</v>
+      </c>
+      <c r="F17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G17" t="s">
+        <v>103</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I17" t="s">
+        <v>46</v>
+      </c>
+      <c r="J17" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="K17" t="s">
+        <v>101</v>
+      </c>
+      <c r="L17" s="4">
+        <v>100</v>
+      </c>
+      <c r="M17" s="4">
+        <v>900</v>
+      </c>
+      <c r="N17" s="4">
+        <v>369</v>
+      </c>
+      <c r="O17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="5:5" x14ac:dyDescent="0.35">
-      <c r="E18" t="s">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="E19" t="s">
         <v>89</v>
       </c>
     </row>

</xml_diff>

<commit_message>
run for shift mid master
</commit_message>
<xml_diff>
--- a/src/test/resources/ExcelResultsFolder/Cards.xlsx
+++ b/src/test/resources/ExcelResultsFolder/Cards.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\git\Integration\src\test\resources\ExcelResultsFolder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{307FF7EE-B607-4902-8677-5FB3C7D0E8F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A1E3CA2-2029-438D-BBB6-404A1474224F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="534" uniqueCount="123">
   <si>
     <t>Matrix</t>
   </si>
@@ -398,6 +398,21 @@
   </si>
   <si>
     <t>4176660000000134</t>
+  </si>
+  <si>
+    <t>5204730000001011</t>
+  </si>
+  <si>
+    <t>5299910010000015</t>
+  </si>
+  <si>
+    <t>5299990270000392</t>
+  </si>
+  <si>
+    <t>5299990270000368</t>
+  </si>
+  <si>
+    <t>5299990270000590</t>
   </si>
 </sst>
 </file>
@@ -826,7 +841,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A047734-60A8-451A-B92F-500542A01A48}">
-  <dimension ref="A1:O23"/>
+  <dimension ref="A1:O28"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.36328125" style="18" customWidth="1"/>
@@ -1736,7 +1751,7 @@
         <v>999</v>
       </c>
       <c r="O19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.35">
@@ -1783,7 +1798,7 @@
         <v>999</v>
       </c>
       <c r="O20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.35">
@@ -1830,7 +1845,7 @@
         <v>999</v>
       </c>
       <c r="O21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.35">
@@ -1877,7 +1892,7 @@
         <v>999</v>
       </c>
       <c r="O22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.35">
@@ -1924,6 +1939,241 @@
         <v>999</v>
       </c>
       <c r="O23" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A24" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E24" t="s">
+        <v>111</v>
+      </c>
+      <c r="F24" t="s">
+        <v>12</v>
+      </c>
+      <c r="G24" t="s">
+        <v>21</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I24" t="s">
+        <v>46</v>
+      </c>
+      <c r="J24" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="K24" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="L24" s="4">
+        <v>100</v>
+      </c>
+      <c r="M24" s="4">
+        <v>900</v>
+      </c>
+      <c r="N24" s="4">
+        <v>249</v>
+      </c>
+      <c r="O24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A25" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E25" t="s">
+        <v>111</v>
+      </c>
+      <c r="F25" t="s">
+        <v>12</v>
+      </c>
+      <c r="G25" t="s">
+        <v>21</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I25" t="s">
+        <v>46</v>
+      </c>
+      <c r="J25" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="K25" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="L25" s="4">
+        <v>100</v>
+      </c>
+      <c r="M25" s="4">
+        <v>900</v>
+      </c>
+      <c r="N25" s="4">
+        <v>249</v>
+      </c>
+      <c r="O25" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A26" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E26" t="s">
+        <v>111</v>
+      </c>
+      <c r="F26" t="s">
+        <v>12</v>
+      </c>
+      <c r="G26" t="s">
+        <v>21</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I26" t="s">
+        <v>46</v>
+      </c>
+      <c r="J26" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="K26" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="L26" s="4">
+        <v>100</v>
+      </c>
+      <c r="M26" s="4">
+        <v>900</v>
+      </c>
+      <c r="N26" s="4">
+        <v>249</v>
+      </c>
+      <c r="O26" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A27" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E27" t="s">
+        <v>111</v>
+      </c>
+      <c r="F27" t="s">
+        <v>12</v>
+      </c>
+      <c r="G27" t="s">
+        <v>21</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I27" t="s">
+        <v>46</v>
+      </c>
+      <c r="J27" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="K27" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="L27" s="4">
+        <v>100</v>
+      </c>
+      <c r="M27" s="4">
+        <v>900</v>
+      </c>
+      <c r="N27" s="4">
+        <v>249</v>
+      </c>
+      <c r="O27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A28" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E28" t="s">
+        <v>111</v>
+      </c>
+      <c r="F28" t="s">
+        <v>16</v>
+      </c>
+      <c r="G28" t="s">
+        <v>21</v>
+      </c>
+      <c r="H28" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I28" t="s">
+        <v>46</v>
+      </c>
+      <c r="J28" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="K28" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="L28" s="4">
+        <v>100</v>
+      </c>
+      <c r="M28" s="4">
+        <v>900</v>
+      </c>
+      <c r="N28" s="4">
+        <v>249</v>
+      </c>
+      <c r="O28" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
master is applied on the shift4
</commit_message>
<xml_diff>
--- a/src/test/resources/ExcelResultsFolder/Cards.xlsx
+++ b/src/test/resources/ExcelResultsFolder/Cards.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\git\Integration\src\test\resources\ExcelResultsFolder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A1E3CA2-2029-438D-BBB6-404A1474224F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{574F9C53-1443-4D5D-8D85-A135A98FEA22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1959,7 +1959,7 @@
         <v>111</v>
       </c>
       <c r="F24" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G24" t="s">
         <v>21</v>
@@ -2006,7 +2006,7 @@
         <v>111</v>
       </c>
       <c r="F25" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G25" t="s">
         <v>21</v>
@@ -2053,7 +2053,7 @@
         <v>111</v>
       </c>
       <c r="F26" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G26" t="s">
         <v>21</v>
@@ -2100,7 +2100,7 @@
         <v>111</v>
       </c>
       <c r="F27" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G27" t="s">
         <v>21</v>

</xml_diff>

<commit_message>
run for payaza card
</commit_message>
<xml_diff>
--- a/src/test/resources/ExcelResultsFolder/Cards.xlsx
+++ b/src/test/resources/ExcelResultsFolder/Cards.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\git\Integration\src\test\resources\ExcelResultsFolder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{574F9C53-1443-4D5D-8D85-A135A98FEA22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AD576AB-836C-4773-AAEB-39E50160FCEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="534" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="126">
   <si>
     <t>Matrix</t>
   </si>
@@ -413,6 +413,15 @@
   </si>
   <si>
     <t>5299990270000590</t>
+  </si>
+  <si>
+    <t>4012000033330026</t>
+  </si>
+  <si>
+    <t>payaza-card</t>
+  </si>
+  <si>
+    <t>NGN</t>
   </si>
 </sst>
 </file>
@@ -841,7 +850,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A047734-60A8-451A-B92F-500542A01A48}">
-  <dimension ref="A1:O28"/>
+  <dimension ref="A1:O30"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.36328125" style="18" customWidth="1"/>
@@ -1986,7 +1995,7 @@
         <v>249</v>
       </c>
       <c r="O24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.35">
@@ -2033,7 +2042,7 @@
         <v>249</v>
       </c>
       <c r="O25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.35">
@@ -2080,7 +2089,7 @@
         <v>249</v>
       </c>
       <c r="O26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.35">
@@ -2127,7 +2136,7 @@
         <v>249</v>
       </c>
       <c r="O27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.35">
@@ -2174,6 +2183,100 @@
         <v>249</v>
       </c>
       <c r="O28" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A29" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="E29" t="s">
+        <v>124</v>
+      </c>
+      <c r="F29" t="s">
+        <v>12</v>
+      </c>
+      <c r="G29" t="s">
+        <v>125</v>
+      </c>
+      <c r="H29" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I29" t="s">
+        <v>46</v>
+      </c>
+      <c r="J29" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="K29" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="L29" s="4">
+        <v>100</v>
+      </c>
+      <c r="M29" s="4">
+        <v>900</v>
+      </c>
+      <c r="N29" s="4">
+        <v>249</v>
+      </c>
+      <c r="O29" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A30" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="E30" t="s">
+        <v>124</v>
+      </c>
+      <c r="F30" t="s">
+        <v>12</v>
+      </c>
+      <c r="G30" t="s">
+        <v>125</v>
+      </c>
+      <c r="H30" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I30" t="s">
+        <v>46</v>
+      </c>
+      <c r="J30" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="K30" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="L30" s="4">
+        <v>100</v>
+      </c>
+      <c r="M30" s="4">
+        <v>900</v>
+      </c>
+      <c r="N30" s="4">
+        <v>249</v>
+      </c>
+      <c r="O30" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
start automation on the sbx
</commit_message>
<xml_diff>
--- a/src/test/resources/ExcelResultsFolder/Cards.xlsx
+++ b/src/test/resources/ExcelResultsFolder/Cards.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\git\Integration\src\test\resources\ExcelResultsFolder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AD576AB-836C-4773-AAEB-39E50160FCEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A8A9D31-1278-4B44-B617-AA8D85B6EA5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="129">
   <si>
     <t>Matrix</t>
   </si>
@@ -422,6 +422,15 @@
   </si>
   <si>
     <t>NGN</t>
+  </si>
+  <si>
+    <t>payable-pix</t>
+  </si>
+  <si>
+    <t>4149011500000147</t>
+  </si>
+  <si>
+    <t>Hazma Sher A Baloch</t>
   </si>
 </sst>
 </file>
@@ -850,7 +859,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A047734-60A8-451A-B92F-500542A01A48}">
-  <dimension ref="A1:O30"/>
+  <dimension ref="A1:O31"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.36328125" style="18" customWidth="1"/>
@@ -2230,7 +2239,7 @@
         <v>249</v>
       </c>
       <c r="O29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.35">
@@ -2277,6 +2286,53 @@
         <v>249</v>
       </c>
       <c r="O30" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A31" s="18" t="s">
+        <v>128</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="E31" t="s">
+        <v>126</v>
+      </c>
+      <c r="F31" t="s">
+        <v>12</v>
+      </c>
+      <c r="G31" t="s">
+        <v>21</v>
+      </c>
+      <c r="H31" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I31" t="s">
+        <v>46</v>
+      </c>
+      <c r="J31" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="K31" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="L31" s="4">
+        <v>1</v>
+      </c>
+      <c r="M31" s="4">
+        <v>2500</v>
+      </c>
+      <c r="N31" s="4">
+        <v>999</v>
+      </c>
+      <c r="O31" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
run for payable sbx
</commit_message>
<xml_diff>
--- a/src/test/resources/ExcelResultsFolder/Cards.xlsx
+++ b/src/test/resources/ExcelResultsFolder/Cards.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\git\Integration\src\test\resources\ExcelResultsFolder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A8A9D31-1278-4B44-B617-AA8D85B6EA5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AA10BC9-65B8-46A8-866A-917E34B0881F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="677" uniqueCount="150">
   <si>
     <t>Matrix</t>
   </si>
@@ -430,7 +430,70 @@
     <t>4149011500000147</t>
   </si>
   <si>
-    <t>Hazma Sher A Baloch</t>
+    <t>5232050000010003</t>
+  </si>
+  <si>
+    <t>Hamza Sher A Baloch</t>
+  </si>
+  <si>
+    <t>4024007119078466</t>
+  </si>
+  <si>
+    <t>4532904789286871</t>
+  </si>
+  <si>
+    <t>12/30</t>
+  </si>
+  <si>
+    <t>4012001037484447</t>
+  </si>
+  <si>
+    <t>12/31</t>
+  </si>
+  <si>
+    <t>124</t>
+  </si>
+  <si>
+    <t>12/32</t>
+  </si>
+  <si>
+    <t>125</t>
+  </si>
+  <si>
+    <t>4012001037461114</t>
+  </si>
+  <si>
+    <t>4242000000000000</t>
+  </si>
+  <si>
+    <t>4012001038443335</t>
+  </si>
+  <si>
+    <t>12/33</t>
+  </si>
+  <si>
+    <t>126</t>
+  </si>
+  <si>
+    <t>12/34</t>
+  </si>
+  <si>
+    <t>127</t>
+  </si>
+  <si>
+    <t>12/35</t>
+  </si>
+  <si>
+    <t>128</t>
+  </si>
+  <si>
+    <t>4242424242420000</t>
+  </si>
+  <si>
+    <t>4012001038488884</t>
+  </si>
+  <si>
+    <t>4242426790614587</t>
   </si>
 </sst>
 </file>
@@ -859,7 +922,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A047734-60A8-451A-B92F-500542A01A48}">
-  <dimension ref="A1:O31"/>
+  <dimension ref="A1:O41"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.36328125" style="18" customWidth="1"/>
@@ -2291,16 +2354,16 @@
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A31" s="18" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>127</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>99</v>
+        <v>66</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>98</v>
+        <v>67</v>
       </c>
       <c r="E31" t="s">
         <v>126</v>
@@ -2320,8 +2383,8 @@
       <c r="J31" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="K31" s="15" t="s">
-        <v>114</v>
+      <c r="K31" t="s">
+        <v>126</v>
       </c>
       <c r="L31" s="4">
         <v>1</v>
@@ -2333,6 +2396,476 @@
         <v>999</v>
       </c>
       <c r="O31" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A32" s="18" t="s">
+        <v>129</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E32" t="s">
+        <v>126</v>
+      </c>
+      <c r="F32" t="s">
+        <v>16</v>
+      </c>
+      <c r="G32" t="s">
+        <v>21</v>
+      </c>
+      <c r="H32" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I32" t="s">
+        <v>46</v>
+      </c>
+      <c r="J32" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="K32" t="s">
+        <v>126</v>
+      </c>
+      <c r="L32" s="4">
+        <v>1</v>
+      </c>
+      <c r="M32" s="4">
+        <v>2500</v>
+      </c>
+      <c r="N32" s="4">
+        <v>999</v>
+      </c>
+      <c r="O32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A33" s="18" t="s">
+        <v>129</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E33" t="s">
+        <v>126</v>
+      </c>
+      <c r="F33" t="s">
+        <v>12</v>
+      </c>
+      <c r="G33" t="s">
+        <v>21</v>
+      </c>
+      <c r="H33" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I33" t="s">
+        <v>46</v>
+      </c>
+      <c r="J33" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="K33" t="s">
+        <v>126</v>
+      </c>
+      <c r="L33" s="4">
+        <v>1</v>
+      </c>
+      <c r="M33" s="4">
+        <v>2500</v>
+      </c>
+      <c r="N33" s="4">
+        <v>999</v>
+      </c>
+      <c r="O33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A34" s="18" t="s">
+        <v>129</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E34" t="s">
+        <v>126</v>
+      </c>
+      <c r="F34" t="s">
+        <v>12</v>
+      </c>
+      <c r="G34" t="s">
+        <v>21</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I34" t="s">
+        <v>46</v>
+      </c>
+      <c r="J34" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="K34" t="s">
+        <v>126</v>
+      </c>
+      <c r="L34" s="4">
+        <v>1</v>
+      </c>
+      <c r="M34" s="4">
+        <v>2500</v>
+      </c>
+      <c r="N34" s="4">
+        <v>999</v>
+      </c>
+      <c r="O34" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A35" s="18" t="s">
+        <v>129</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E35" t="s">
+        <v>126</v>
+      </c>
+      <c r="F35" t="s">
+        <v>12</v>
+      </c>
+      <c r="G35" t="s">
+        <v>21</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I35" t="s">
+        <v>46</v>
+      </c>
+      <c r="J35" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="K35" t="s">
+        <v>126</v>
+      </c>
+      <c r="L35" s="4">
+        <v>1</v>
+      </c>
+      <c r="M35" s="4">
+        <v>2500</v>
+      </c>
+      <c r="N35" s="4">
+        <v>249</v>
+      </c>
+      <c r="O35" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A36" s="18" t="s">
+        <v>129</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E36" t="s">
+        <v>126</v>
+      </c>
+      <c r="F36" t="s">
+        <v>12</v>
+      </c>
+      <c r="G36" t="s">
+        <v>21</v>
+      </c>
+      <c r="H36" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I36" t="s">
+        <v>46</v>
+      </c>
+      <c r="J36" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="K36" t="s">
+        <v>126</v>
+      </c>
+      <c r="L36" s="4">
+        <v>1</v>
+      </c>
+      <c r="M36" s="4">
+        <v>2500</v>
+      </c>
+      <c r="N36" s="4">
+        <v>249</v>
+      </c>
+      <c r="O36" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A37" s="18" t="s">
+        <v>129</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="D37" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="E37" t="s">
+        <v>126</v>
+      </c>
+      <c r="F37" t="s">
+        <v>12</v>
+      </c>
+      <c r="G37" t="s">
+        <v>21</v>
+      </c>
+      <c r="H37" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I37" t="s">
+        <v>46</v>
+      </c>
+      <c r="J37" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="K37" t="s">
+        <v>126</v>
+      </c>
+      <c r="L37" s="4">
+        <v>1</v>
+      </c>
+      <c r="M37" s="4">
+        <v>2500</v>
+      </c>
+      <c r="N37" s="4">
+        <v>249</v>
+      </c>
+      <c r="O37" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A38" s="18" t="s">
+        <v>129</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="D38" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="E38" t="s">
+        <v>126</v>
+      </c>
+      <c r="F38" t="s">
+        <v>12</v>
+      </c>
+      <c r="G38" t="s">
+        <v>21</v>
+      </c>
+      <c r="H38" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I38" t="s">
+        <v>46</v>
+      </c>
+      <c r="J38" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="K38" t="s">
+        <v>126</v>
+      </c>
+      <c r="L38" s="4">
+        <v>1</v>
+      </c>
+      <c r="M38" s="4">
+        <v>2500</v>
+      </c>
+      <c r="N38" s="4">
+        <v>249</v>
+      </c>
+      <c r="O38" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A39" s="18" t="s">
+        <v>129</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="E39" t="s">
+        <v>126</v>
+      </c>
+      <c r="F39" t="s">
+        <v>12</v>
+      </c>
+      <c r="G39" t="s">
+        <v>21</v>
+      </c>
+      <c r="H39" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I39" t="s">
+        <v>46</v>
+      </c>
+      <c r="J39" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="K39" t="s">
+        <v>126</v>
+      </c>
+      <c r="L39" s="4">
+        <v>1</v>
+      </c>
+      <c r="M39" s="4">
+        <v>2500</v>
+      </c>
+      <c r="N39" s="4">
+        <v>249</v>
+      </c>
+      <c r="O39" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A40" s="18" t="s">
+        <v>129</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="E40" t="s">
+        <v>126</v>
+      </c>
+      <c r="F40" t="s">
+        <v>12</v>
+      </c>
+      <c r="G40" t="s">
+        <v>21</v>
+      </c>
+      <c r="H40" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I40" t="s">
+        <v>46</v>
+      </c>
+      <c r="J40" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="K40" t="s">
+        <v>126</v>
+      </c>
+      <c r="L40" s="4">
+        <v>1</v>
+      </c>
+      <c r="M40" s="4">
+        <v>2500</v>
+      </c>
+      <c r="N40" s="4">
+        <v>249</v>
+      </c>
+      <c r="O40" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A41" s="18" t="s">
+        <v>129</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="E41" t="s">
+        <v>126</v>
+      </c>
+      <c r="F41" t="s">
+        <v>12</v>
+      </c>
+      <c r="G41" t="s">
+        <v>21</v>
+      </c>
+      <c r="H41" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I41" t="s">
+        <v>46</v>
+      </c>
+      <c r="J41" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="K41" t="s">
+        <v>126</v>
+      </c>
+      <c r="L41" s="4">
+        <v>1</v>
+      </c>
+      <c r="M41" s="4">
+        <v>2500</v>
+      </c>
+      <c r="N41" s="4">
+        <v>249</v>
+      </c>
+      <c r="O41" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
run for yoya pay payin
</commit_message>
<xml_diff>
--- a/src/test/resources/ExcelResultsFolder/Cards.xlsx
+++ b/src/test/resources/ExcelResultsFolder/Cards.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\git\Integration\src\test\resources\ExcelResultsFolder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23631A34-75CF-466D-81CD-DE5FE35C79B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{767E25A5-9BD9-4AB4-8FE1-DECDFF0DFAFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="710" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="732" uniqueCount="154">
   <si>
     <t>Matrix</t>
   </si>
@@ -497,6 +497,15 @@
   </si>
   <si>
     <t>5454545454545454</t>
+  </si>
+  <si>
+    <t>5200000000000015</t>
+  </si>
+  <si>
+    <t>yoyapayPayin</t>
+  </si>
+  <si>
+    <t>Test Test</t>
   </si>
 </sst>
 </file>
@@ -924,7 +933,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A047734-60A8-451A-B92F-500542A01A48}">
-  <dimension ref="A1:O44"/>
+  <dimension ref="A1:O46"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.36328125" style="17" customWidth="1"/>
@@ -2398,7 +2407,7 @@
         <v>999</v>
       </c>
       <c r="O31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.35">
@@ -3010,6 +3019,100 @@
       </c>
       <c r="O44" t="b">
         <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A45" s="17" t="s">
+        <v>127</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="E45" t="s">
+        <v>124</v>
+      </c>
+      <c r="F45" t="s">
+        <v>16</v>
+      </c>
+      <c r="G45" t="s">
+        <v>70</v>
+      </c>
+      <c r="H45" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I45" t="s">
+        <v>46</v>
+      </c>
+      <c r="J45" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="K45" t="s">
+        <v>124</v>
+      </c>
+      <c r="L45" s="4">
+        <v>1</v>
+      </c>
+      <c r="M45" s="4">
+        <v>2500</v>
+      </c>
+      <c r="N45" s="4">
+        <v>249</v>
+      </c>
+      <c r="O45" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A46" s="17" t="s">
+        <v>153</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="D46" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E46" t="s">
+        <v>152</v>
+      </c>
+      <c r="F46" t="s">
+        <v>12</v>
+      </c>
+      <c r="G46" t="s">
+        <v>21</v>
+      </c>
+      <c r="H46" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I46" t="s">
+        <v>46</v>
+      </c>
+      <c r="J46" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="K46" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="L46" s="4">
+        <v>1</v>
+      </c>
+      <c r="M46" s="4">
+        <v>2500</v>
+      </c>
+      <c r="N46" s="4">
+        <v>123</v>
+      </c>
+      <c r="O46" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
change card for yoyapaypayin
</commit_message>
<xml_diff>
--- a/src/test/resources/ExcelResultsFolder/Cards.xlsx
+++ b/src/test/resources/ExcelResultsFolder/Cards.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\git\Integration\src\test\resources\ExcelResultsFolder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{767E25A5-9BD9-4AB4-8FE1-DECDFF0DFAFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33CE1772-D6AA-42BC-A363-9D45B799D22C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3073,7 +3073,7 @@
         <v>153</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>9</v>
+        <v>103</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>130</v>

</xml_diff>